<commit_message>
Feat: mostrar todos los datos del cliente en ResultPanel (frontend)
- Reemplaza grid de 4 campos por tabla completa con 13 variables
- Muestra política crediticia, propósito, tasa, cuota, ingreso real,
  FICO, DTI, días crédito, balance revolving, utilización, consultas,
  morosidades y registros públicos
- Ingreso convertido de log a valor real con Math.exp()
- Filas alternadas para mejor legibilidad

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/clientes_prueba.xlsx
+++ b/clientes_prueba.xlsx
@@ -463,31 +463,31 @@
         <v>debt_consolidation</v>
       </c>
       <c r="C2">
-        <v>0.1189</v>
+        <v>0.08</v>
       </c>
       <c r="D2">
-        <v>366.86</v>
+        <v>300.5</v>
       </c>
       <c r="E2">
-        <v>11.35</v>
+        <v>11.8</v>
       </c>
       <c r="F2">
-        <v>19.48</v>
+        <v>12.5</v>
       </c>
       <c r="G2">
-        <v>737</v>
+        <v>780</v>
       </c>
       <c r="H2">
-        <v>5639.96</v>
+        <v>6500</v>
       </c>
       <c r="I2">
-        <v>28854</v>
+        <v>15000</v>
       </c>
       <c r="J2">
-        <v>52.1</v>
+        <v>30</v>
       </c>
       <c r="K2">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L2">
         <v>0</v>
@@ -504,28 +504,28 @@
         <v>credit_card</v>
       </c>
       <c r="C3">
-        <v>0.1008</v>
+        <v>0.095</v>
       </c>
       <c r="D3">
         <v>162.34</v>
       </c>
       <c r="E3">
-        <v>11.08</v>
+        <v>11.35</v>
       </c>
       <c r="F3">
-        <v>16.29</v>
+        <v>16.3</v>
       </c>
       <c r="G3">
-        <v>742</v>
+        <v>760</v>
       </c>
       <c r="H3">
-        <v>4200</v>
+        <v>5600</v>
       </c>
       <c r="I3">
-        <v>15000</v>
+        <v>12000</v>
       </c>
       <c r="J3">
-        <v>30.5</v>
+        <v>22</v>
       </c>
       <c r="K3">
         <v>0</v>
@@ -545,7 +545,7 @@
         <v>home_improvement</v>
       </c>
       <c r="C4">
-        <v>0.09</v>
+        <v>0.085</v>
       </c>
       <c r="D4">
         <v>215</v>
@@ -557,16 +557,16 @@
         <v>10</v>
       </c>
       <c r="G4">
-        <v>780</v>
+        <v>800</v>
       </c>
       <c r="H4">
-        <v>6500</v>
+        <v>7000</v>
       </c>
       <c r="I4">
-        <v>10000</v>
+        <v>8000</v>
       </c>
       <c r="J4">
-        <v>18</v>
+        <v>15</v>
       </c>
       <c r="K4">
         <v>0</v>
@@ -586,28 +586,28 @@
         <v>major_purchase</v>
       </c>
       <c r="C5">
-        <v>0.095</v>
+        <v>0.105</v>
       </c>
       <c r="D5">
-        <v>300</v>
+        <v>280</v>
       </c>
       <c r="E5">
         <v>11.2</v>
       </c>
       <c r="F5">
-        <v>12.5</v>
+        <v>14</v>
       </c>
       <c r="G5">
-        <v>760</v>
+        <v>740</v>
       </c>
       <c r="H5">
-        <v>5800</v>
+        <v>5200</v>
       </c>
       <c r="I5">
-        <v>8000</v>
+        <v>9000</v>
       </c>
       <c r="J5">
-        <v>22</v>
+        <v>28</v>
       </c>
       <c r="K5">
         <v>1</v>
@@ -627,28 +627,28 @@
         <v>educational</v>
       </c>
       <c r="C6">
-        <v>0.105</v>
+        <v>0.11</v>
       </c>
       <c r="D6">
-        <v>180.5</v>
+        <v>190</v>
       </c>
       <c r="E6">
         <v>10.9</v>
       </c>
       <c r="F6">
-        <v>14</v>
+        <v>13.5</v>
       </c>
       <c r="G6">
-        <v>715</v>
+        <v>725</v>
       </c>
       <c r="H6">
-        <v>3650</v>
+        <v>4000</v>
       </c>
       <c r="I6">
         <v>5000</v>
       </c>
       <c r="J6">
-        <v>25</v>
+        <v>20</v>
       </c>
       <c r="K6">
         <v>0</v>
@@ -662,122 +662,122 @@
     </row>
     <row r="7">
       <c r="A7">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="B7" t="str">
         <v>debt_consolidation</v>
       </c>
       <c r="C7">
-        <v>0.1357</v>
+        <v>0.2</v>
       </c>
       <c r="D7">
-        <v>450</v>
+        <v>500</v>
       </c>
       <c r="E7">
-        <v>10.8</v>
+        <v>10.2</v>
       </c>
       <c r="F7">
-        <v>28.5</v>
+        <v>38</v>
       </c>
       <c r="G7">
-        <v>680</v>
+        <v>620</v>
       </c>
       <c r="H7">
-        <v>3200</v>
+        <v>2000</v>
       </c>
       <c r="I7">
-        <v>22000</v>
+        <v>30000</v>
       </c>
       <c r="J7">
-        <v>55</v>
+        <v>72</v>
       </c>
       <c r="K7">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="L7">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M7">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="8">
       <c r="A8">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="B8" t="str">
         <v>small_business</v>
       </c>
       <c r="C8">
-        <v>0.15</v>
+        <v>0.22</v>
       </c>
       <c r="D8">
-        <v>520</v>
+        <v>580</v>
       </c>
       <c r="E8">
-        <v>10.7</v>
+        <v>10.1</v>
       </c>
       <c r="F8">
-        <v>32</v>
+        <v>42</v>
       </c>
       <c r="G8">
-        <v>660</v>
+        <v>600</v>
       </c>
       <c r="H8">
-        <v>2900</v>
+        <v>1800</v>
       </c>
       <c r="I8">
-        <v>18000</v>
+        <v>35000</v>
       </c>
       <c r="J8">
-        <v>62</v>
+        <v>78</v>
       </c>
       <c r="K8">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="L8">
         <v>1</v>
       </c>
       <c r="M8">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="9">
       <c r="A9">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="B9" t="str">
         <v>credit_card</v>
       </c>
       <c r="C9">
-        <v>0.1299</v>
+        <v>0.19</v>
       </c>
       <c r="D9">
-        <v>380</v>
+        <v>460</v>
       </c>
       <c r="E9">
-        <v>10.6</v>
+        <v>10.3</v>
       </c>
       <c r="F9">
-        <v>25</v>
+        <v>35</v>
       </c>
       <c r="G9">
-        <v>695</v>
+        <v>640</v>
       </c>
       <c r="H9">
-        <v>4100</v>
+        <v>2200</v>
       </c>
       <c r="I9">
-        <v>20000</v>
+        <v>28000</v>
       </c>
       <c r="J9">
-        <v>48</v>
+        <v>68</v>
       </c>
       <c r="K9">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="L9">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M9">
         <v>0</v>
@@ -788,31 +788,31 @@
         <v>0</v>
       </c>
       <c r="B10" t="str">
-        <v>home_improvement</v>
+        <v>all_other</v>
       </c>
       <c r="C10">
-        <v>0.145</v>
+        <v>0.21</v>
       </c>
       <c r="D10">
-        <v>410</v>
+        <v>540</v>
       </c>
       <c r="E10">
-        <v>10.9</v>
+        <v>10</v>
       </c>
       <c r="F10">
-        <v>30</v>
+        <v>40</v>
       </c>
       <c r="G10">
-        <v>670</v>
+        <v>610</v>
       </c>
       <c r="H10">
-        <v>3500</v>
+        <v>1600</v>
       </c>
       <c r="I10">
-        <v>25000</v>
+        <v>32000</v>
       </c>
       <c r="J10">
-        <v>58</v>
+        <v>75</v>
       </c>
       <c r="K10">
         <v>1</v>
@@ -821,48 +821,48 @@
         <v>1</v>
       </c>
       <c r="M10">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="11">
       <c r="A11">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="B11" t="str">
-        <v>major_purchase</v>
+        <v>home_improvement</v>
       </c>
       <c r="C11">
-        <v>0.138</v>
+        <v>0.23</v>
       </c>
       <c r="D11">
-        <v>295</v>
+        <v>620</v>
       </c>
       <c r="E11">
-        <v>10.5</v>
+        <v>10.15</v>
       </c>
       <c r="F11">
-        <v>27</v>
+        <v>44</v>
       </c>
       <c r="G11">
-        <v>688</v>
+        <v>595</v>
       </c>
       <c r="H11">
-        <v>2800</v>
+        <v>1500</v>
       </c>
       <c r="I11">
-        <v>12000</v>
+        <v>38000</v>
       </c>
       <c r="J11">
-        <v>44</v>
+        <v>80</v>
       </c>
       <c r="K11">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="L11">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M11">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="12">
@@ -873,34 +873,34 @@
         <v>debt_consolidation</v>
       </c>
       <c r="C12">
-        <v>0.199</v>
+        <v>0.55</v>
       </c>
       <c r="D12">
-        <v>650</v>
+        <v>1200</v>
       </c>
       <c r="E12">
-        <v>10.2</v>
+        <v>8.5</v>
       </c>
       <c r="F12">
-        <v>45</v>
+        <v>65</v>
       </c>
       <c r="G12">
-        <v>590</v>
+        <v>350</v>
       </c>
       <c r="H12">
-        <v>1800</v>
+        <v>300</v>
       </c>
       <c r="I12">
-        <v>35000</v>
+        <v>80000</v>
       </c>
       <c r="J12">
-        <v>82</v>
+        <v>99</v>
       </c>
       <c r="K12">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="L12">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="M12">
         <v>1</v>
@@ -914,37 +914,37 @@
         <v>small_business</v>
       </c>
       <c r="C13">
-        <v>0.21</v>
+        <v>0.6</v>
       </c>
       <c r="D13">
-        <v>720</v>
+        <v>1400</v>
       </c>
       <c r="E13">
-        <v>10</v>
+        <v>8.2</v>
       </c>
       <c r="F13">
-        <v>48</v>
+        <v>70</v>
       </c>
       <c r="G13">
-        <v>560</v>
+        <v>320</v>
       </c>
       <c r="H13">
-        <v>1500</v>
+        <v>200</v>
       </c>
       <c r="I13">
-        <v>40000</v>
+        <v>90000</v>
       </c>
       <c r="J13">
-        <v>90</v>
+        <v>99</v>
       </c>
       <c r="K13">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="L13">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="M13">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="14">
@@ -955,34 +955,34 @@
         <v>all_other</v>
       </c>
       <c r="C14">
-        <v>0.22</v>
+        <v>0.7</v>
       </c>
       <c r="D14">
-        <v>580</v>
+        <v>1600</v>
       </c>
       <c r="E14">
-        <v>10.1</v>
+        <v>8</v>
       </c>
       <c r="F14">
-        <v>50</v>
+        <v>75</v>
       </c>
       <c r="G14">
-        <v>545</v>
+        <v>300</v>
       </c>
       <c r="H14">
-        <v>1200</v>
+        <v>100</v>
       </c>
       <c r="I14">
-        <v>32000</v>
+        <v>95000</v>
       </c>
       <c r="J14">
-        <v>88</v>
+        <v>99</v>
       </c>
       <c r="K14">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="L14">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="M14">
         <v>1</v>
@@ -996,34 +996,34 @@
         <v>credit_card</v>
       </c>
       <c r="C15">
-        <v>0.195</v>
+        <v>0.58</v>
       </c>
       <c r="D15">
-        <v>500</v>
+        <v>1300</v>
       </c>
       <c r="E15">
-        <v>10.3</v>
+        <v>8.3</v>
       </c>
       <c r="F15">
-        <v>43</v>
+        <v>68</v>
       </c>
       <c r="G15">
-        <v>610</v>
+        <v>330</v>
       </c>
       <c r="H15">
-        <v>2000</v>
+        <v>250</v>
       </c>
       <c r="I15">
-        <v>28000</v>
+        <v>85000</v>
       </c>
       <c r="J15">
-        <v>78</v>
+        <v>99</v>
       </c>
       <c r="K15">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="L15">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="M15">
         <v>1</v>
@@ -1037,37 +1037,37 @@
         <v>debt_consolidation</v>
       </c>
       <c r="C16">
-        <v>0.205</v>
+        <v>0.65</v>
       </c>
       <c r="D16">
-        <v>690</v>
+        <v>1500</v>
       </c>
       <c r="E16">
-        <v>9.9</v>
+        <v>8.1</v>
       </c>
       <c r="F16">
-        <v>52</v>
+        <v>72</v>
       </c>
       <c r="G16">
-        <v>530</v>
+        <v>310</v>
       </c>
       <c r="H16">
-        <v>1100</v>
+        <v>150</v>
       </c>
       <c r="I16">
-        <v>45000</v>
+        <v>92000</v>
       </c>
       <c r="J16">
-        <v>95</v>
+        <v>99</v>
       </c>
       <c r="K16">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="L16">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="M16">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
   </sheetData>

</xml_diff>